<commit_message>
Quality Assessment: update completed
</commit_message>
<xml_diff>
--- a/data/literature/bib/quality-assessment/analysis.xlsx
+++ b/data/literature/bib/quality-assessment/analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sousa\Dev\phd-trp\data\literature\bib\quality-assessment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929B15A7-A004-4511-ACF6-70C8ECF0658E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE15A76-4346-4991-949E-26629033EE3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Eligible Records" sheetId="1" r:id="rId1"/>
@@ -19,10 +19,10 @@
     <sheet name="Graphs Analysis" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Analysis!$C$28:$C$48</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Analysis!$D$28:$D$48</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Analysis!$C$2:$C$22</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Analysis!$D$2:$D$22</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Analysis!$C$2:$C$22</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Analysis!$D$2:$D$22</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Analysis!$C$28:$C$48</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Analysis!$D$28:$D$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,6 +38,208 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Ricardo Barbosa Sousa</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{4F2461D3-C286-48F5-BD93-A91CCE9150BF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dynamic</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A9" authorId="0" shapeId="0" xr:uid="{84B39B30-172A-46E4-88B9-8E9C4D90C5E2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dynamic</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A10" authorId="0" shapeId="0" xr:uid="{64AF61A8-4C65-4BCF-9DD0-F0E3EAD739A7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dynamic</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{AB03A520-74E8-4FF9-85A2-F3E5768EE292}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dynamic</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A13" authorId="0" shapeId="0" xr:uid="{459E4F5C-E2A5-47DB-96AA-479CCD1D24EB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dynamic</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{39DA9295-4666-4829-B52B-E6BEB05DBA67}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Seems to be an extension of the 2 other works from Berrio!</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A27" authorId="0" shapeId="0" xr:uid="{B7A70068-6692-4331-88CC-2CE824635816}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+already in the SLR</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A28" authorId="0" shapeId="0" xr:uid="{D17749AB-CB39-4B01-B3D8-EA3107D6BCED}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Ricardo Barbosa Sousa:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+not available</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
@@ -63,7 +265,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="385">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="385">
   <si>
     <t>title</t>
   </si>
@@ -1256,7 +1458,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1301,6 +1503,19 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1356,9 +1571,6 @@
   </cellStyles>
   <dxfs count="51">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -1412,9 +1624,6 @@
           <bgColor rgb="FFE2EFDA"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
@@ -1538,6 +1747,12 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -2052,10 +2267,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v1.2</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.3</cx:f>
+        <cx:f>_xlchart.v1.1</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2266,10 +2481,10 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:strDim type="cat">
-        <cx:f>_xlchart.v1.0</cx:f>
+        <cx:f>_xlchart.v1.2</cx:f>
       </cx:strDim>
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.3</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -3620,8 +3835,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="320040" y="167640"/>
-              <a:ext cx="4888523" cy="2834640"/>
+              <a:off x="314325" y="161925"/>
+              <a:ext cx="4802798" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3698,8 +3913,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5760720" y="167640"/>
-              <a:ext cx="4888523" cy="2834640"/>
+              <a:off x="5657850" y="161925"/>
+              <a:ext cx="4802798" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3773,8 +3988,8 @@
     <tableColumn id="12" xr3:uid="{0F077A71-3EE7-490D-B55E-70827DE813E8}" name="author"/>
     <tableColumn id="13" xr3:uid="{E81C4977-098C-4325-9C40-73E84C0ED44B}" name="year"/>
     <tableColumn id="19" xr3:uid="{46BD9103-423C-4179-B05A-B3E5ED93DB26}" name="doi" dataDxfId="32"/>
-    <tableColumn id="18" xr3:uid="{54F3D085-288F-444A-B63F-9ECE6012AB45}" name="url" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{2BCE0B96-9C49-403C-B867-209A2FBEA6A6}" name="QE parsifal" dataDxfId="8">
+    <tableColumn id="18" xr3:uid="{54F3D085-288F-444A-B63F-9ECE6012AB45}" name="url" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{2BCE0B96-9C49-403C-B867-209A2FBEA6A6}" name="QE parsifal" dataDxfId="30">
       <calculatedColumnFormula>Table2[[#This Row],[QE score]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{9AA448D7-C56A-4D11-92A3-DF2ED2805C05}" name="QE1: related"/>
@@ -3785,16 +4000,16 @@
     <tableColumn id="8" xr3:uid="{3BF21DF8-1E1C-487B-9808-0878BAFE5257}" name="QE6: others"/>
     <tableColumn id="3" xr3:uid="{54B0E2A3-CBA0-4064-BAA1-3F6098448B2E}" name="QE7: public"/>
     <tableColumn id="4" xr3:uid="{D0C73622-DB34-495D-AE54-B520D304E58D}" name="QE8: results"/>
-    <tableColumn id="5" xr3:uid="{CD562DBB-99FE-43D9-A9CE-AE17C5B42CE8}" name="QE score" dataDxfId="31">
+    <tableColumn id="5" xr3:uid="{CD562DBB-99FE-43D9-A9CE-AE17C5B42CE8}" name="QE score" dataDxfId="29">
       <calculatedColumnFormula>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{08CFC487-1911-4523-B4F7-08D3704EBCB5}" name="QE R1:_x000a_QE2/3/5/8" dataDxfId="30">
+    <tableColumn id="16" xr3:uid="{08CFC487-1911-4523-B4F7-08D3704EBCB5}" name="QE R1:_x000a_QE2/3/5/8" dataDxfId="28">
       <calculatedColumnFormula>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{146DE30D-BAE5-4D76-BDC1-96A99DD6A808}" name="QE R2:_x000a_cut-off" dataDxfId="29">
+    <tableColumn id="14" xr3:uid="{146DE30D-BAE5-4D76-BDC1-96A99DD6A808}" name="QE R2:_x000a_cut-off" dataDxfId="27">
       <calculatedColumnFormula>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{A6EA9EB1-7A33-482B-AD2C-06AB5AFB4F94}" name="include?" dataDxfId="28">
+    <tableColumn id="17" xr3:uid="{A6EA9EB1-7A33-482B-AD2C-06AB5AFB4F94}" name="include?" dataDxfId="26">
       <calculatedColumnFormula>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</calculatedColumnFormula>
@@ -3805,21 +4020,21 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D216FC5C-BC08-42D4-B4E1-15413C03FFAD}" name="Table4" displayName="Table4" ref="A1:A4" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{D216FC5C-BC08-42D4-B4E1-15413C03FFAD}" name="Table4" displayName="Table4" ref="A1:A4" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="A1:A4" xr:uid="{D216FC5C-BC08-42D4-B4E1-15413C03FFAD}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{BFB27CC8-6784-4A15-9BE3-FC016698C653}" name="QE options" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{BFB27CC8-6784-4A15-9BE3-FC016698C653}" name="QE options" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CC8D7A7E-57EA-48C7-8BE2-5733263DD580}" name="Table3" displayName="Table3" ref="C1:D22" totalsRowShown="0" headerRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CC8D7A7E-57EA-48C7-8BE2-5733263DD580}" name="Table3" displayName="Table3" ref="C1:D22" totalsRowShown="0" headerRowDxfId="22">
   <autoFilter ref="C1:D22" xr:uid="{CC8D7A7E-57EA-48C7-8BE2-5733263DD580}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{536DF366-6912-4F71-946E-28E7190508D7}" name="QE scores"/>
-    <tableColumn id="2" xr3:uid="{240223F8-A5E3-481C-B7A6-C0256D4044C0}" name="#records" dataDxfId="23">
+    <tableColumn id="2" xr3:uid="{240223F8-A5E3-481C-B7A6-C0256D4044C0}" name="#records" dataDxfId="21">
       <calculatedColumnFormula>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3828,17 +4043,17 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{84295ABF-7A89-4807-9E44-78F7C46DF235}" name="Table5" displayName="Table5" ref="L1:N22" totalsRowShown="0" headerRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{84295ABF-7A89-4807-9E44-78F7C46DF235}" name="Table5" displayName="Table5" ref="L1:N22" totalsRowShown="0" headerRowDxfId="20">
   <autoFilter ref="L1:N22" xr:uid="{84295ABF-7A89-4807-9E44-78F7C46DF235}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="L2:M22">
     <sortCondition descending="1" ref="L1:L22"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{4DA02C84-0999-4962-A444-6B4204A5E049}" name="QE scores"/>
-    <tableColumn id="2" xr3:uid="{15021F80-EA71-4DDC-982C-22B79CEE6582}" name="cumul #" dataDxfId="21">
+    <tableColumn id="2" xr3:uid="{15021F80-EA71-4DDC-982C-22B79CEE6582}" name="cumul #" dataDxfId="19">
       <calculatedColumnFormula>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{D1006D37-E3B1-4616-B9B1-F5CCBCE714E7}" name="%" dataDxfId="20">
+    <tableColumn id="3" xr3:uid="{D1006D37-E3B1-4616-B9B1-F5CCBCE714E7}" name="%" dataDxfId="18">
       <calculatedColumnFormula>Table5[[#This Row],[cumul '#]]/$D$23</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3847,41 +4062,41 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A88E6F42-C0FC-4197-8315-AA79C16EC324}" name="Table37" displayName="Table37" ref="C27:M48" totalsRowShown="0" headerRowDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A88E6F42-C0FC-4197-8315-AA79C16EC324}" name="Table37" displayName="Table37" ref="C27:M48" totalsRowShown="0" headerRowDxfId="17">
   <autoFilter ref="C27:M48" xr:uid="{A88E6F42-C0FC-4197-8315-AA79C16EC324}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{EF6AE36E-B85B-426F-9EDD-16C88C3EE827}" name="QE scores"/>
-    <tableColumn id="2" xr3:uid="{1F708127-0EE7-45C3-9781-227B95252131}" name="#records" dataDxfId="18">
+    <tableColumn id="2" xr3:uid="{1F708127-0EE7-45C3-9781-227B95252131}" name="#records" dataDxfId="16">
       <calculatedColumnFormula>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{08BE139C-68C7-4863-A278-D110ABA9B2B3}" name="cumul #" dataDxfId="17">
+    <tableColumn id="3" xr3:uid="{08BE139C-68C7-4863-A278-D110ABA9B2B3}" name="cumul #" dataDxfId="15">
       <calculatedColumnFormula>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{5D112F35-304D-4446-A0BC-8DF2DDEBE096}" name="%cumul #" dataDxfId="16">
+    <tableColumn id="7" xr3:uid="{5D112F35-304D-4446-A0BC-8DF2DDEBE096}" name="%cumul #" dataDxfId="14">
       <calculatedColumnFormula>Table37[[#This Row],[cumul '#]]/$D$49</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{810A7296-E2E8-4E2B-A332-D6331CAD791E}" name="%cumul # total" dataDxfId="15">
+    <tableColumn id="12" xr3:uid="{810A7296-E2E8-4E2B-A332-D6331CAD791E}" name="%cumul # total" dataDxfId="13">
       <calculatedColumnFormula>Table37[[#This Row],[cumul '#]]/$D$23</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{71DE376A-A25E-47E8-A802-39F2519D4438}" name="inv cuml #" dataDxfId="14">
+    <tableColumn id="13" xr3:uid="{71DE376A-A25E-47E8-A802-39F2519D4438}" name="inv cuml #" dataDxfId="12">
       <calculatedColumnFormula>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{CE0FFC32-19D8-478B-97C1-C6E06ED4EFFB}" name="%inv cuml #" dataDxfId="13">
+    <tableColumn id="14" xr3:uid="{CE0FFC32-19D8-478B-97C1-C6E06ED4EFFB}" name="%inv cuml #" dataDxfId="11">
       <calculatedColumnFormula>Table37[[#This Row],[inv cuml '#]]/$D$49</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0CA2304A-D741-4509-A1B7-C00BE206837E}" name="Y" dataDxfId="12">
+    <tableColumn id="8" xr3:uid="{0CA2304A-D741-4509-A1B7-C00BE206837E}" name="Y" dataDxfId="10">
       <calculatedColumnFormula>Table37[[#This Row],['#records]]/$D$49</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2509A1D1-46B5-4A44-AF15-23D6B6BD15F2}" name="^Y" dataDxfId="11">
+    <tableColumn id="9" xr3:uid="{2509A1D1-46B5-4A44-AF15-23D6B6BD15F2}" name="^Y" dataDxfId="9">
       <calculatedColumnFormula>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{F9102C1E-598A-4E76-8CCA-04F1C1E23915}" name="^#records" dataDxfId="10">
+    <tableColumn id="10" xr3:uid="{F9102C1E-598A-4E76-8CCA-04F1C1E23915}" name="^#records" dataDxfId="8">
       <calculatedColumnFormula>Table37[[#This Row],[^Y]]*$D$49</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BCE9461F-1944-4EF6-9406-247DC53831DA}" name="error" dataDxfId="9">
+    <tableColumn id="11" xr3:uid="{BCE9461F-1944-4EF6-9406-247DC53831DA}" name="error" dataDxfId="7">
       <calculatedColumnFormula>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4190,26 +4405,26 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:P30"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="70.6640625" customWidth="1"/>
+    <col min="1" max="1" width="70.7109375" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="9.5546875" customWidth="1"/>
-    <col min="4" max="4" width="7.88671875" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" customWidth="1"/>
-    <col min="6" max="6" width="8.5546875" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" customWidth="1"/>
+    <col min="4" max="4" width="7.85546875" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="11.6640625" customWidth="1"/>
-    <col min="13" max="13" width="18.5546875" customWidth="1"/>
-    <col min="14" max="14" width="11.6640625" customWidth="1"/>
-    <col min="15" max="15" width="11.5546875" customWidth="1"/>
-    <col min="16" max="16" width="7.88671875" customWidth="1"/>
+    <col min="10" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" customWidth="1"/>
+    <col min="13" max="13" width="18.5703125" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" customWidth="1"/>
+    <col min="16" max="16" width="7.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4259,7 +4474,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>130</v>
       </c>
@@ -4297,7 +4512,7 @@
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>138</v>
       </c>
@@ -4339,7 +4554,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>63</v>
       </c>
@@ -4389,7 +4604,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>148</v>
       </c>
@@ -4439,7 +4654,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>158</v>
       </c>
@@ -4485,7 +4700,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>166</v>
       </c>
@@ -4535,7 +4750,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -4585,7 +4800,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>180</v>
       </c>
@@ -4635,7 +4850,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>192</v>
       </c>
@@ -4681,7 +4896,7 @@
       </c>
       <c r="P10" s="2"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>201</v>
       </c>
@@ -4731,7 +4946,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>210</v>
       </c>
@@ -4775,7 +4990,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>219</v>
       </c>
@@ -4825,7 +5040,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>227</v>
       </c>
@@ -4875,7 +5090,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>236</v>
       </c>
@@ -4925,7 +5140,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>245</v>
       </c>
@@ -4969,7 +5184,7 @@
       </c>
       <c r="P16" s="2"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>254</v>
       </c>
@@ -5019,7 +5234,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>264</v>
       </c>
@@ -5069,7 +5284,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>273</v>
       </c>
@@ -5119,7 +5334,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>282</v>
       </c>
@@ -5169,7 +5384,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>291</v>
       </c>
@@ -5215,7 +5430,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>299</v>
       </c>
@@ -5261,7 +5476,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>307</v>
       </c>
@@ -5311,7 +5526,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>318</v>
       </c>
@@ -5361,7 +5576,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>331</v>
       </c>
@@ -5403,7 +5618,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>338</v>
       </c>
@@ -5441,7 +5656,7 @@
       <c r="O26" s="2"/>
       <c r="P26" s="2"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>345</v>
       </c>
@@ -5485,7 +5700,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>36</v>
       </c>
@@ -5521,7 +5736,7 @@
       </c>
       <c r="P28" s="2"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>30</v>
       </c>
@@ -5557,7 +5772,7 @@
       </c>
       <c r="P29" s="2"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>354</v>
       </c>
@@ -5608,19 +5823,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7545F806-0EAB-4CC4-B735-EF2845EB43B6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7545F806-0EAB-4CC4-B735-EF2845EB43B6}">
   <dimension ref="A1:R31"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="50.6640625" customWidth="1"/>
-    <col min="2" max="2" width="20.6640625" customWidth="1"/>
-    <col min="3" max="5" width="8.33203125" customWidth="1"/>
-    <col min="6" max="15" width="13.33203125" customWidth="1"/>
-    <col min="16" max="17" width="13.44140625" customWidth="1"/>
-    <col min="18" max="18" width="13.33203125" customWidth="1"/>
+    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="3" max="5" width="8.28515625" customWidth="1"/>
+    <col min="6" max="15" width="13.28515625" customWidth="1"/>
+    <col min="16" max="17" width="13.42578125" customWidth="1"/>
+    <col min="18" max="18" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="F1" s="3" t="s">
         <v>95</v>
       </c>
@@ -5655,7 +5870,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -5711,29 +5926,53 @@
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>148</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>149</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="F3">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3" t="s">
+        <v>92</v>
+      </c>
+      <c r="I3" t="s">
+        <v>93</v>
+      </c>
+      <c r="J3" t="s">
+        <v>92</v>
+      </c>
+      <c r="K3" t="s">
+        <v>92</v>
+      </c>
+      <c r="L3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" t="s">
+        <v>92</v>
+      </c>
+      <c r="N3" t="s">
+        <v>92</v>
       </c>
       <c r="O3">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P3" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5741,38 +5980,62 @@
       </c>
       <c r="Q3" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R3" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>236</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>237</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>142</v>
+        <v>240</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="F4">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8.5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H4" t="s">
+        <v>92</v>
+      </c>
+      <c r="I4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J4" t="s">
+        <v>92</v>
+      </c>
+      <c r="K4" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M4" t="s">
+        <v>94</v>
+      </c>
+      <c r="N4" t="s">
+        <v>92</v>
       </c>
       <c r="O4">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="P4" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5780,38 +6043,62 @@
       </c>
       <c r="Q4" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R4" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>318</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>319</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>54</v>
+        <v>324</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="F5">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H5" t="s">
+        <v>92</v>
+      </c>
+      <c r="I5" t="s">
+        <v>92</v>
+      </c>
+      <c r="J5" t="s">
+        <v>93</v>
+      </c>
+      <c r="K5" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" t="s">
+        <v>92</v>
+      </c>
+      <c r="M5" t="s">
+        <v>92</v>
+      </c>
+      <c r="N5" t="s">
+        <v>92</v>
       </c>
       <c r="O5">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P5" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5819,38 +6106,62 @@
       </c>
       <c r="Q5" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R5" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>299</v>
       </c>
       <c r="B6" t="s">
-        <v>149</v>
+        <v>300</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>153</v>
+        <v>303</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="F6">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8.5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6" t="s">
+        <v>92</v>
+      </c>
+      <c r="I6" t="s">
+        <v>93</v>
+      </c>
+      <c r="J6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K6" t="s">
+        <v>92</v>
+      </c>
+      <c r="L6" t="s">
+        <v>92</v>
+      </c>
+      <c r="M6" t="s">
+        <v>92</v>
+      </c>
+      <c r="N6" t="s">
+        <v>92</v>
       </c>
       <c r="O6">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="P6" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5858,38 +6169,62 @@
       </c>
       <c r="Q6" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R6" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>282</v>
       </c>
       <c r="B7" t="s">
-        <v>159</v>
+        <v>283</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>162</v>
+        <v>286</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="F7">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8.5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H7" t="s">
+        <v>93</v>
+      </c>
+      <c r="I7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J7" t="s">
+        <v>93</v>
+      </c>
+      <c r="K7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L7" t="s">
+        <v>92</v>
+      </c>
+      <c r="M7" t="s">
+        <v>92</v>
+      </c>
+      <c r="N7" t="s">
+        <v>92</v>
       </c>
       <c r="O7">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="P7" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5897,38 +6232,62 @@
       </c>
       <c r="Q7" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R7" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>166</v>
+        <v>130</v>
       </c>
       <c r="B8" t="s">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>170</v>
+        <v>135</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="F8">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8.5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>93</v>
+      </c>
+      <c r="H8" t="s">
+        <v>92</v>
+      </c>
+      <c r="I8" t="s">
+        <v>93</v>
+      </c>
+      <c r="J8" t="s">
+        <v>92</v>
+      </c>
+      <c r="K8" t="s">
+        <v>92</v>
+      </c>
+      <c r="L8" t="s">
+        <v>92</v>
+      </c>
+      <c r="M8" t="s">
+        <v>92</v>
+      </c>
+      <c r="N8" t="s">
+        <v>92</v>
       </c>
       <c r="O8">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="P8" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5936,38 +6295,62 @@
       </c>
       <c r="Q8" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R8" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>192</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>193</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>28</v>
+        <v>196</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F9">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" t="s">
+        <v>92</v>
+      </c>
+      <c r="I9" t="s">
+        <v>92</v>
+      </c>
+      <c r="J9" t="s">
+        <v>93</v>
+      </c>
+      <c r="K9" t="s">
+        <v>92</v>
+      </c>
+      <c r="L9" t="s">
+        <v>92</v>
+      </c>
+      <c r="M9" t="s">
+        <v>94</v>
+      </c>
+      <c r="N9" t="s">
+        <v>93</v>
       </c>
       <c r="O9">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P9" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -5975,38 +6358,62 @@
       </c>
       <c r="Q9" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R9" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>180</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>181</v>
+        <v>31</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>186</v>
+        <v>33</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>371</v>
+        <v>353</v>
       </c>
       <c r="F10">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8.5</v>
+      </c>
+      <c r="G10" t="s">
+        <v>93</v>
+      </c>
+      <c r="H10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I10" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" t="s">
+        <v>93</v>
+      </c>
+      <c r="K10" t="s">
+        <v>92</v>
+      </c>
+      <c r="L10" t="s">
+        <v>92</v>
+      </c>
+      <c r="M10" t="s">
+        <v>92</v>
+      </c>
+      <c r="N10" t="s">
+        <v>93</v>
       </c>
       <c r="O10">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="P10" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6014,38 +6421,62 @@
       </c>
       <c r="Q10" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R10" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>192</v>
+        <v>307</v>
       </c>
       <c r="B11" t="s">
-        <v>193</v>
+        <v>308</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>196</v>
+        <v>312</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="F11">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8.5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>93</v>
+      </c>
+      <c r="H11" t="s">
+        <v>92</v>
+      </c>
+      <c r="I11" t="s">
+        <v>93</v>
+      </c>
+      <c r="J11" t="s">
+        <v>92</v>
+      </c>
+      <c r="K11" t="s">
+        <v>92</v>
+      </c>
+      <c r="L11" t="s">
+        <v>92</v>
+      </c>
+      <c r="M11" t="s">
+        <v>92</v>
+      </c>
+      <c r="N11" t="s">
+        <v>92</v>
       </c>
       <c r="O11">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8.5</v>
       </c>
       <c r="P11" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6053,38 +6484,62 @@
       </c>
       <c r="Q11" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R11" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>201</v>
+        <v>354</v>
       </c>
       <c r="B12" t="s">
-        <v>202</v>
+        <v>355</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>205</v>
+        <v>358</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="F12">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="G12" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" t="s">
+        <v>92</v>
+      </c>
+      <c r="I12" t="s">
+        <v>93</v>
+      </c>
+      <c r="J12" t="s">
+        <v>92</v>
+      </c>
+      <c r="K12" t="s">
+        <v>92</v>
+      </c>
+      <c r="L12" t="s">
+        <v>92</v>
+      </c>
+      <c r="M12" t="s">
+        <v>94</v>
+      </c>
+      <c r="N12" t="s">
+        <v>92</v>
       </c>
       <c r="O12">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P12" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6092,38 +6547,62 @@
       </c>
       <c r="Q12" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R12" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>210</v>
+        <v>273</v>
       </c>
       <c r="B13" t="s">
-        <v>211</v>
+        <v>274</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>216</v>
+        <v>277</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="F13">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="G13" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" t="s">
+        <v>92</v>
+      </c>
+      <c r="I13" t="s">
+        <v>93</v>
+      </c>
+      <c r="J13" t="s">
+        <v>92</v>
+      </c>
+      <c r="K13" t="s">
+        <v>92</v>
+      </c>
+      <c r="L13" t="s">
+        <v>92</v>
+      </c>
+      <c r="M13" t="s">
+        <v>92</v>
+      </c>
+      <c r="N13" t="s">
+        <v>92</v>
       </c>
       <c r="O13">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="P13" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6131,38 +6610,62 @@
       </c>
       <c r="Q13" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R13" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>219</v>
+        <v>138</v>
       </c>
       <c r="B14" t="s">
-        <v>220</v>
+        <v>139</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>222</v>
+        <v>142</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="F14">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>9.5</v>
+      </c>
+      <c r="G14" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" t="s">
+        <v>93</v>
+      </c>
+      <c r="I14" t="s">
+        <v>92</v>
+      </c>
+      <c r="J14" t="s">
+        <v>92</v>
+      </c>
+      <c r="K14" t="s">
+        <v>92</v>
+      </c>
+      <c r="L14" t="s">
+        <v>92</v>
+      </c>
+      <c r="M14" t="s">
+        <v>92</v>
+      </c>
+      <c r="N14" t="s">
+        <v>92</v>
       </c>
       <c r="O14">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="P14" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6170,38 +6673,62 @@
       </c>
       <c r="Q14" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R14" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>227</v>
+        <v>264</v>
       </c>
       <c r="B15" t="s">
-        <v>228</v>
+        <v>265</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>231</v>
+        <v>268</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="F15">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="G15" t="s">
+        <v>94</v>
+      </c>
+      <c r="H15" t="s">
+        <v>93</v>
+      </c>
+      <c r="I15" t="s">
+        <v>92</v>
+      </c>
+      <c r="J15" t="s">
+        <v>92</v>
+      </c>
+      <c r="K15" t="s">
+        <v>92</v>
+      </c>
+      <c r="L15" t="s">
+        <v>92</v>
+      </c>
+      <c r="M15" t="s">
+        <v>92</v>
+      </c>
+      <c r="N15" t="s">
+        <v>93</v>
       </c>
       <c r="O15">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="P15" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6209,38 +6736,62 @@
       </c>
       <c r="Q15" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
-        <v>reject</v>
+        <v>ok</v>
       </c>
       <c r="R15" s="5" t="str">
         <f>IF(AND(Table2[[#This Row],[QE R1:
 QE2/3/5/8]] &lt;&gt; "reject", Table2[[#This Row],[QE R2:
 cut-off]] &lt;&gt; "reject"),"yes","no")</f>
-        <v>no</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+        <v>yes</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>236</v>
+        <v>180</v>
       </c>
       <c r="B16" t="s">
-        <v>237</v>
+        <v>181</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>240</v>
+        <v>186</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="F16">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7.5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>94</v>
+      </c>
+      <c r="H16" t="s">
+        <v>93</v>
+      </c>
+      <c r="I16" t="s">
+        <v>92</v>
+      </c>
+      <c r="J16" t="s">
+        <v>93</v>
+      </c>
+      <c r="K16" t="s">
+        <v>92</v>
+      </c>
+      <c r="L16" t="s">
+        <v>92</v>
+      </c>
+      <c r="M16" t="s">
+        <v>92</v>
+      </c>
+      <c r="N16" t="s">
+        <v>93</v>
       </c>
       <c r="O16">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="P16" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6257,33 +6808,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>245</v>
+        <v>345</v>
       </c>
       <c r="B17" t="s">
-        <v>246</v>
+        <v>46</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>250</v>
+        <v>48</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>378</v>
+        <v>348</v>
       </c>
       <c r="F17">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="G17" t="s">
+        <v>93</v>
+      </c>
+      <c r="H17" t="s">
+        <v>93</v>
+      </c>
+      <c r="I17" t="s">
+        <v>92</v>
+      </c>
+      <c r="J17" t="s">
+        <v>93</v>
+      </c>
+      <c r="K17" t="s">
+        <v>94</v>
+      </c>
+      <c r="L17" t="s">
+        <v>92</v>
+      </c>
+      <c r="M17" t="s">
+        <v>94</v>
+      </c>
+      <c r="N17" t="s">
+        <v>93</v>
       </c>
       <c r="O17">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="P17" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q17" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6296,29 +6871,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>254</v>
+        <v>166</v>
       </c>
       <c r="B18" t="s">
-        <v>255</v>
+        <v>167</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>259</v>
+        <v>170</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="F18">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7.5</v>
+      </c>
+      <c r="G18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H18" t="s">
+        <v>93</v>
+      </c>
+      <c r="I18" t="s">
+        <v>93</v>
+      </c>
+      <c r="J18" t="s">
+        <v>93</v>
+      </c>
+      <c r="K18" t="s">
+        <v>92</v>
+      </c>
+      <c r="L18" t="s">
+        <v>92</v>
+      </c>
+      <c r="M18" t="s">
+        <v>92</v>
+      </c>
+      <c r="N18" t="s">
+        <v>93</v>
       </c>
       <c r="O18">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="P18" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6335,33 +6934,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="B19" t="s">
-        <v>265</v>
+        <v>246</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="F19">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="G19" t="s">
+        <v>94</v>
+      </c>
+      <c r="H19" t="s">
+        <v>94</v>
+      </c>
+      <c r="I19" t="s">
+        <v>93</v>
+      </c>
+      <c r="J19" t="s">
+        <v>92</v>
+      </c>
+      <c r="K19" t="s">
+        <v>94</v>
+      </c>
+      <c r="L19" t="s">
+        <v>92</v>
+      </c>
+      <c r="M19" t="s">
+        <v>94</v>
+      </c>
+      <c r="N19" t="s">
+        <v>94</v>
       </c>
       <c r="O19">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P19" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q19" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6374,29 +6997,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>273</v>
+        <v>210</v>
       </c>
       <c r="B20" t="s">
-        <v>274</v>
+        <v>211</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>277</v>
+        <v>216</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>381</v>
+        <v>374</v>
       </c>
       <c r="F20">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="G20" t="s">
+        <v>94</v>
+      </c>
+      <c r="H20" t="s">
+        <v>93</v>
+      </c>
+      <c r="I20" t="s">
+        <v>93</v>
+      </c>
+      <c r="J20" t="s">
+        <v>92</v>
+      </c>
+      <c r="K20" t="s">
+        <v>92</v>
+      </c>
+      <c r="L20" t="s">
+        <v>92</v>
+      </c>
+      <c r="M20" t="s">
+        <v>92</v>
+      </c>
+      <c r="N20" t="s">
+        <v>93</v>
       </c>
       <c r="O20">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P20" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6413,33 +7060,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>282</v>
+        <v>338</v>
       </c>
       <c r="B21" t="s">
-        <v>283</v>
+        <v>339</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>286</v>
+        <v>343</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>362</v>
+        <v>384</v>
       </c>
       <c r="F21">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="G21" t="s">
+        <v>93</v>
+      </c>
+      <c r="H21" t="s">
+        <v>93</v>
+      </c>
+      <c r="I21" t="s">
+        <v>92</v>
+      </c>
+      <c r="J21" t="s">
+        <v>92</v>
+      </c>
+      <c r="K21" t="s">
+        <v>94</v>
+      </c>
+      <c r="L21" t="s">
+        <v>92</v>
+      </c>
+      <c r="M21" t="s">
+        <v>92</v>
+      </c>
+      <c r="N21" t="s">
+        <v>92</v>
       </c>
       <c r="O21">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P21" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q21" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6452,29 +7123,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>291</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>292</v>
+        <v>26</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>295</v>
+        <v>28</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="F22">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7.5</v>
+      </c>
+      <c r="G22" t="s">
+        <v>92</v>
+      </c>
+      <c r="H22" t="s">
+        <v>92</v>
+      </c>
+      <c r="I22" t="s">
+        <v>93</v>
+      </c>
+      <c r="J22" t="s">
+        <v>92</v>
+      </c>
+      <c r="K22" t="s">
+        <v>92</v>
+      </c>
+      <c r="L22" t="s">
+        <v>94</v>
+      </c>
+      <c r="M22" t="s">
+        <v>92</v>
+      </c>
+      <c r="N22" t="s">
+        <v>93</v>
       </c>
       <c r="O22">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="P22" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6491,29 +7186,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>299</v>
+        <v>158</v>
       </c>
       <c r="B23" t="s">
-        <v>300</v>
+        <v>159</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>303</v>
+        <v>162</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F23">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7.5</v>
+      </c>
+      <c r="G23" t="s">
+        <v>93</v>
+      </c>
+      <c r="H23" t="s">
+        <v>92</v>
+      </c>
+      <c r="I23" t="s">
+        <v>93</v>
+      </c>
+      <c r="J23" t="s">
+        <v>93</v>
+      </c>
+      <c r="K23" t="s">
+        <v>92</v>
+      </c>
+      <c r="L23" t="s">
+        <v>92</v>
+      </c>
+      <c r="M23" t="s">
+        <v>92</v>
+      </c>
+      <c r="N23" t="s">
+        <v>93</v>
       </c>
       <c r="O23">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="P23" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6530,29 +7249,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="B24" t="s">
-        <v>308</v>
+        <v>292</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>312</v>
+        <v>295</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="F24">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>6.5</v>
+      </c>
+      <c r="G24" t="s">
+        <v>94</v>
+      </c>
+      <c r="H24" t="s">
+        <v>93</v>
+      </c>
+      <c r="I24" t="s">
+        <v>92</v>
+      </c>
+      <c r="J24" t="s">
+        <v>93</v>
+      </c>
+      <c r="K24" t="s">
+        <v>92</v>
+      </c>
+      <c r="L24" t="s">
+        <v>92</v>
+      </c>
+      <c r="M24" t="s">
+        <v>94</v>
+      </c>
+      <c r="N24" t="s">
+        <v>93</v>
       </c>
       <c r="O24">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>6.5</v>
       </c>
       <c r="P24" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6569,33 +7312,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>318</v>
+        <v>219</v>
       </c>
       <c r="B25" t="s">
-        <v>319</v>
+        <v>220</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>324</v>
+        <v>222</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>382</v>
+        <v>375</v>
       </c>
       <c r="F25">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="G25" t="s">
+        <v>94</v>
+      </c>
+      <c r="H25" t="s">
+        <v>94</v>
+      </c>
+      <c r="I25" t="s">
+        <v>92</v>
+      </c>
+      <c r="J25" t="s">
+        <v>93</v>
+      </c>
+      <c r="K25" t="s">
+        <v>94</v>
+      </c>
+      <c r="L25" t="s">
+        <v>92</v>
+      </c>
+      <c r="M25" t="s">
+        <v>94</v>
+      </c>
+      <c r="N25" t="s">
+        <v>93</v>
       </c>
       <c r="O25">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P25" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q25" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6608,7 +7375,7 @@
         <v>no</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>331</v>
       </c>
@@ -6626,15 +7393,39 @@
       </c>
       <c r="F26">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="G26" t="s">
+        <v>93</v>
+      </c>
+      <c r="H26" t="s">
+        <v>93</v>
+      </c>
+      <c r="I26" t="s">
+        <v>92</v>
+      </c>
+      <c r="J26" t="s">
+        <v>93</v>
+      </c>
+      <c r="K26" t="s">
+        <v>94</v>
+      </c>
+      <c r="L26" t="s">
+        <v>92</v>
+      </c>
+      <c r="M26" t="s">
+        <v>92</v>
+      </c>
+      <c r="N26" t="s">
+        <v>93</v>
       </c>
       <c r="O26">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P26" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q26" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6647,33 +7438,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>338</v>
+        <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>339</v>
+        <v>37</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>343</v>
+        <v>39</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>384</v>
+        <v>351</v>
       </c>
       <c r="F27">
         <f>Table2[[#This Row],[QE score]]</f>
         <v>0</v>
       </c>
+      <c r="G27" t="s">
+        <v>94</v>
+      </c>
+      <c r="H27" t="s">
+        <v>94</v>
+      </c>
+      <c r="I27" t="s">
+        <v>94</v>
+      </c>
+      <c r="J27" t="s">
+        <v>94</v>
+      </c>
+      <c r="K27" t="s">
+        <v>94</v>
+      </c>
+      <c r="L27" t="s">
+        <v>94</v>
+      </c>
+      <c r="M27" t="s">
+        <v>94</v>
+      </c>
+      <c r="N27" t="s">
+        <v>94</v>
+      </c>
       <c r="O27">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="P27" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q27" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6686,33 +7501,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>345</v>
+        <v>254</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>255</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>48</v>
+        <v>259</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>348</v>
+        <v>379</v>
       </c>
       <c r="F28">
         <f>Table2[[#This Row],[QE score]]</f>
         <v>0</v>
       </c>
+      <c r="G28" t="s">
+        <v>94</v>
+      </c>
+      <c r="H28" t="s">
+        <v>94</v>
+      </c>
+      <c r="I28" t="s">
+        <v>94</v>
+      </c>
+      <c r="J28" t="s">
+        <v>94</v>
+      </c>
+      <c r="K28" t="s">
+        <v>94</v>
+      </c>
+      <c r="L28" t="s">
+        <v>94</v>
+      </c>
+      <c r="M28" t="s">
+        <v>94</v>
+      </c>
+      <c r="N28" t="s">
+        <v>94</v>
+      </c>
       <c r="O28">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
         <v>0</v>
       </c>
       <c r="P28" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q28" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6725,29 +7564,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>201</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>202</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>39</v>
+        <v>205</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>351</v>
+        <v>373</v>
       </c>
       <c r="F29">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="G29" t="s">
+        <v>94</v>
+      </c>
+      <c r="H29" t="s">
+        <v>93</v>
+      </c>
+      <c r="I29" t="s">
+        <v>93</v>
+      </c>
+      <c r="J29" t="s">
+        <v>92</v>
+      </c>
+      <c r="K29" t="s">
+        <v>92</v>
+      </c>
+      <c r="L29" t="s">
+        <v>92</v>
+      </c>
+      <c r="M29" t="s">
+        <v>92</v>
+      </c>
+      <c r="N29" t="s">
+        <v>93</v>
       </c>
       <c r="O29">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="P29" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6764,33 +7627,57 @@
         <v>no</v>
       </c>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>227</v>
       </c>
       <c r="B30" t="s">
-        <v>31</v>
+        <v>228</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>33</v>
+        <v>231</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>353</v>
+        <v>376</v>
       </c>
       <c r="F30">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="G30" t="s">
+        <v>94</v>
+      </c>
+      <c r="H30" t="s">
+        <v>93</v>
+      </c>
+      <c r="I30" t="s">
+        <v>92</v>
+      </c>
+      <c r="J30" t="s">
+        <v>92</v>
+      </c>
+      <c r="K30" t="s">
+        <v>94</v>
+      </c>
+      <c r="L30" t="s">
+        <v>92</v>
+      </c>
+      <c r="M30" t="s">
+        <v>92</v>
+      </c>
+      <c r="N30" t="s">
+        <v>93</v>
       </c>
       <c r="O30">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P30" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
-        <v>ok</v>
+        <v>reject</v>
       </c>
       <c r="Q30" s="5" t="str">
         <f>IF(Table2[[#This Row],[QE score]]&lt;=$Q$1,"reject","ok")</f>
@@ -6803,29 +7690,53 @@
         <v>no</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>354</v>
+        <v>63</v>
       </c>
       <c r="B31" t="s">
-        <v>355</v>
+        <v>53</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>358</v>
+        <v>54</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="F31">
         <f>Table2[[#This Row],[QE score]]</f>
-        <v>0</v>
+        <v>7.5</v>
+      </c>
+      <c r="G31" t="s">
+        <v>93</v>
+      </c>
+      <c r="H31" t="s">
+        <v>93</v>
+      </c>
+      <c r="I31" t="s">
+        <v>92</v>
+      </c>
+      <c r="J31" t="s">
+        <v>92</v>
+      </c>
+      <c r="K31" t="s">
+        <v>92</v>
+      </c>
+      <c r="L31" t="s">
+        <v>92</v>
+      </c>
+      <c r="M31" t="s">
+        <v>94</v>
+      </c>
+      <c r="N31" t="s">
+        <v>93</v>
       </c>
       <c r="O31">
         <f>IF(Table2[[#This Row],[QE1: related]]="full",G$1,IF(Table2[[#This Row],[QE1: related]]="partial",G$1*0.5,0))+IF(Table2[[#This Row],[QE2: method]]="full",H$1,IF(Table2[[#This Row],[QE2: method]]="partial",H$1*0.5,0))+IF(Table2[[#This Row],[QE3: l+m]]="full",I$1,IF(Table2[[#This Row],[QE3: l+m]]="partial",I$1*0.5,0))+IF(Table2[[#This Row],[QE4: hw+sw]]="full",J$1,IF(Table2[[#This Row],[QE4: hw+sw]]="partial",J$1*0.5,0))+IF(Table2[[#This Row],[QE5: long]]="full",K$1,IF(Table2[[#This Row],[QE5: long]]="partial",K$1*0.5,0))+IF(Table2[[#This Row],[QE6: others]]="full",L$1,IF(Table2[[#This Row],[QE6: others]]="partial",L$1*0.5,0))+IF(Table2[[#This Row],[QE7: public]]="full",M$1,IF(Table2[[#This Row],[QE7: public]]="partial",M$1*0.5,0))+IF(Table2[[#This Row],[QE8: results]]="full",N$1,IF(Table2[[#This Row],[QE8: results]]="partial",N$1*0.5,0))</f>
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="P31" t="str">
         <f>IF(OR(Table2[[#This Row],[QE2: method]]="none",Table2[[#This Row],[QE3: l+m]]="none",Table2[[#This Row],[QE5: long]]="none",Table2[[#This Row],[QE8: results]]="none"),"reject","ok")</f>
@@ -6845,69 +7756,70 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="F3:F31">
-    <cfRule type="expression" dxfId="7" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F3=$O3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:N31">
-    <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>"full"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="7" operator="equal">
       <formula>"partial"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="8" operator="equal">
       <formula>"none"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O3:R31">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$R3="yes"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="5">
+    <cfRule type="expression" dxfId="1" priority="5">
       <formula>$R3="no"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:R31">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="0" priority="2">
       <formula>$F3&lt;&gt;$O3</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{C701380C-7362-4FCE-890F-05A1237B6E7E}"/>
-    <hyperlink ref="E4" r:id="rId2" xr:uid="{868A804E-D793-45C4-8C9E-7365B15544B7}"/>
-    <hyperlink ref="E5" r:id="rId3" xr:uid="{8D0A991A-BB8C-480F-8886-5ADF17633836}"/>
-    <hyperlink ref="E6" r:id="rId4" xr:uid="{A0DD27D0-CA36-4CB0-8073-77BB4B3A6098}"/>
-    <hyperlink ref="E7" r:id="rId5" xr:uid="{D4A4BE2B-9DD5-435A-9249-D56AFD480B7C}"/>
-    <hyperlink ref="E8" r:id="rId6" xr:uid="{EFB9915A-7E76-4FBF-92A2-3359780929B5}"/>
-    <hyperlink ref="E9" r:id="rId7" xr:uid="{A6461E8C-25F3-49F4-BE64-9884D3DD6FBF}"/>
-    <hyperlink ref="E10" r:id="rId8" xr:uid="{6A0145BA-A71E-43FD-8546-C62DF03FADE4}"/>
-    <hyperlink ref="E11" r:id="rId9" xr:uid="{0954FADA-A081-4555-881D-26C2C9018669}"/>
-    <hyperlink ref="E12" r:id="rId10" xr:uid="{55DB8388-D16E-4912-AD65-4C33490CA46E}"/>
-    <hyperlink ref="E13" r:id="rId11" xr:uid="{7A13338A-327D-41D0-AA1B-BA491BBF8141}"/>
-    <hyperlink ref="E14" r:id="rId12" xr:uid="{6C95EA31-11B7-4CC9-8AFA-F3AF410F838C}"/>
-    <hyperlink ref="E15" r:id="rId13" xr:uid="{20F4F1EB-3639-449B-9445-D90A33744BB1}"/>
-    <hyperlink ref="E16" r:id="rId14" xr:uid="{2BFFBC0A-5B2D-42AA-92DA-D009BDBDE9F7}"/>
-    <hyperlink ref="E17" r:id="rId15" xr:uid="{CCFFBECD-B20B-41A3-B3EB-F5409E59CDF5}"/>
-    <hyperlink ref="E18" r:id="rId16" xr:uid="{5380D309-9E81-4E4D-8C9C-21DC7152520F}"/>
-    <hyperlink ref="E19" r:id="rId17" xr:uid="{71FEC21B-5406-46CA-977D-2FB3C98384C0}"/>
-    <hyperlink ref="E20" r:id="rId18" xr:uid="{221D605E-537D-48C0-B99C-9BD630803441}"/>
-    <hyperlink ref="E21" r:id="rId19" xr:uid="{4CB16497-66AD-472C-8E4E-A2C1586F7E4D}"/>
-    <hyperlink ref="E22" r:id="rId20" xr:uid="{B4209E08-6A26-4E6C-9849-CA1DB3CC7810}"/>
-    <hyperlink ref="E23" r:id="rId21" xr:uid="{414C0BBB-C8AE-40A9-82BF-F6C519EEB0D6}"/>
-    <hyperlink ref="E24" r:id="rId22" xr:uid="{B415C92C-0A8D-4B4F-ABC0-F692A64E4303}"/>
-    <hyperlink ref="E25" r:id="rId23" xr:uid="{4332E9A0-301A-4295-A4C0-FCF0B27B6CA5}"/>
+    <hyperlink ref="E8" r:id="rId1" xr:uid="{C701380C-7362-4FCE-890F-05A1237B6E7E}"/>
+    <hyperlink ref="E14" r:id="rId2" xr:uid="{868A804E-D793-45C4-8C9E-7365B15544B7}"/>
+    <hyperlink ref="E31" r:id="rId3" xr:uid="{8D0A991A-BB8C-480F-8886-5ADF17633836}"/>
+    <hyperlink ref="E3" r:id="rId4" xr:uid="{A0DD27D0-CA36-4CB0-8073-77BB4B3A6098}"/>
+    <hyperlink ref="E23" r:id="rId5" xr:uid="{D4A4BE2B-9DD5-435A-9249-D56AFD480B7C}"/>
+    <hyperlink ref="E18" r:id="rId6" xr:uid="{EFB9915A-7E76-4FBF-92A2-3359780929B5}"/>
+    <hyperlink ref="E22" r:id="rId7" xr:uid="{A6461E8C-25F3-49F4-BE64-9884D3DD6FBF}"/>
+    <hyperlink ref="E16" r:id="rId8" xr:uid="{6A0145BA-A71E-43FD-8546-C62DF03FADE4}"/>
+    <hyperlink ref="E9" r:id="rId9" xr:uid="{0954FADA-A081-4555-881D-26C2C9018669}"/>
+    <hyperlink ref="E29" r:id="rId10" xr:uid="{55DB8388-D16E-4912-AD65-4C33490CA46E}"/>
+    <hyperlink ref="E20" r:id="rId11" xr:uid="{7A13338A-327D-41D0-AA1B-BA491BBF8141}"/>
+    <hyperlink ref="E25" r:id="rId12" xr:uid="{6C95EA31-11B7-4CC9-8AFA-F3AF410F838C}"/>
+    <hyperlink ref="E30" r:id="rId13" xr:uid="{20F4F1EB-3639-449B-9445-D90A33744BB1}"/>
+    <hyperlink ref="E4" r:id="rId14" xr:uid="{2BFFBC0A-5B2D-42AA-92DA-D009BDBDE9F7}"/>
+    <hyperlink ref="E19" r:id="rId15" xr:uid="{CCFFBECD-B20B-41A3-B3EB-F5409E59CDF5}"/>
+    <hyperlink ref="E28" r:id="rId16" xr:uid="{5380D309-9E81-4E4D-8C9C-21DC7152520F}"/>
+    <hyperlink ref="E15" r:id="rId17" xr:uid="{71FEC21B-5406-46CA-977D-2FB3C98384C0}"/>
+    <hyperlink ref="E13" r:id="rId18" xr:uid="{221D605E-537D-48C0-B99C-9BD630803441}"/>
+    <hyperlink ref="E7" r:id="rId19" xr:uid="{4CB16497-66AD-472C-8E4E-A2C1586F7E4D}"/>
+    <hyperlink ref="E24" r:id="rId20" xr:uid="{B4209E08-6A26-4E6C-9849-CA1DB3CC7810}"/>
+    <hyperlink ref="E6" r:id="rId21" xr:uid="{414C0BBB-C8AE-40A9-82BF-F6C519EEB0D6}"/>
+    <hyperlink ref="E11" r:id="rId22" xr:uid="{B415C92C-0A8D-4B4F-ABC0-F692A64E4303}"/>
+    <hyperlink ref="E5" r:id="rId23" xr:uid="{4332E9A0-301A-4295-A4C0-FCF0B27B6CA5}"/>
     <hyperlink ref="E26" r:id="rId24" xr:uid="{9EE0E5EC-5192-48D6-BA8A-4A42DF2D83F5}"/>
-    <hyperlink ref="E27" r:id="rId25" xr:uid="{039C7DF1-01A1-4931-B656-D5DE945150FA}"/>
-    <hyperlink ref="E28" r:id="rId26" xr:uid="{9C69FA90-10FC-4647-A3EE-CD252B4B125A}"/>
-    <hyperlink ref="E29" r:id="rId27" xr:uid="{A3EF606F-C0F9-412D-9C43-AF354555F90A}"/>
-    <hyperlink ref="E30" r:id="rId28" xr:uid="{40FBCED4-9660-4263-8F36-209CB3B3C733}"/>
-    <hyperlink ref="E31" r:id="rId29" xr:uid="{E345D5AD-92C5-447F-9377-C22A16DED340}"/>
+    <hyperlink ref="E21" r:id="rId25" xr:uid="{039C7DF1-01A1-4931-B656-D5DE945150FA}"/>
+    <hyperlink ref="E17" r:id="rId26" xr:uid="{9C69FA90-10FC-4647-A3EE-CD252B4B125A}"/>
+    <hyperlink ref="E27" r:id="rId27" xr:uid="{A3EF606F-C0F9-412D-9C43-AF354555F90A}"/>
+    <hyperlink ref="E10" r:id="rId28" xr:uid="{40FBCED4-9660-4263-8F36-209CB3B3C733}"/>
+    <hyperlink ref="E12" r:id="rId29" xr:uid="{E345D5AD-92C5-447F-9377-C22A16DED340}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
+  <legacyDrawing r:id="rId31"/>
   <tableParts count="1">
-    <tablePart r:id="rId31"/>
+    <tablePart r:id="rId32"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -6927,22 +7839,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4CC010-3585-447F-ACB4-C01A0F7A7EBA}">
   <dimension ref="A1:P52"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.77734375" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.88671875" customWidth="1"/>
-    <col min="12" max="12" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.85546875" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>91</v>
       </c>
@@ -6965,7 +7877,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>92</v>
       </c>
@@ -6974,7 +7886,7 @@
       </c>
       <c r="D2">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>100</v>
@@ -6994,7 +7906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>93</v>
       </c>
@@ -7010,14 +7922,14 @@
       </c>
       <c r="M3">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N3" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+        <v>3.4482758620689655E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>94</v>
       </c>
@@ -7036,14 +7948,14 @@
       </c>
       <c r="M4">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N4" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.13793103448275862</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C5">
         <v>1.5</v>
       </c>
@@ -7056,25 +7968,25 @@
       </c>
       <c r="I5">
         <f>SUMIF(Table3[QE scores],"&gt;"&amp;$I$2,Table3['#records])</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J5" s="9">
         <f>I5/SUM(Table3['#records])</f>
-        <v>0</v>
+        <v>0.44827586206896552</v>
       </c>
       <c r="L5">
         <v>8.5</v>
       </c>
       <c r="M5">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="N5" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.34482758620689657</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C6">
         <v>2</v>
       </c>
@@ -7087,25 +7999,25 @@
       </c>
       <c r="I6">
         <f>SUMIF(Table3[QE scores],"&lt;="&amp;$I$2,Table3['#records])</f>
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="J6" s="9">
         <f>I6/SUM(Table3['#records])</f>
-        <v>1</v>
+        <v>0.55172413793103448</v>
       </c>
       <c r="L6">
         <v>8</v>
       </c>
       <c r="M6">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="N6" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.44827586206896552</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C7">
         <v>2.5</v>
       </c>
@@ -7118,20 +8030,20 @@
       </c>
       <c r="M7">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="N7" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.62068965517241381</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C8">
         <v>3</v>
       </c>
       <c r="D8">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>107</v>
@@ -7141,14 +8053,14 @@
       </c>
       <c r="M8">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="N8" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.72413793103448276</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C9">
         <v>3.5</v>
       </c>
@@ -7161,56 +8073,56 @@
       </c>
       <c r="I9">
         <f>COUNTIF(Table2[include?],"=yes")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J9" s="9">
         <f>I9/SUM(Table3['#records])</f>
-        <v>0</v>
+        <v>0.44827586206896552</v>
       </c>
       <c r="L9">
         <v>6.5</v>
       </c>
       <c r="M9">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="N9" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.75862068965517238</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C10">
         <v>4</v>
       </c>
       <c r="D10">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>101</v>
       </c>
       <c r="I10">
         <f>I12+I11</f>
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="J10" s="9">
         <f>I10/SUM(Table3['#records])</f>
-        <v>1</v>
+        <v>0.55172413793103448</v>
       </c>
       <c r="L10">
         <v>6</v>
       </c>
       <c r="M10">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N10" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.82758620689655171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C11">
         <v>4.5</v>
       </c>
@@ -7224,31 +8136,31 @@
       <c r="I11">
         <f>COUNTIF(Table2[QE R1:
 QE2/3/5/8],"reject")</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J11" s="9">
         <f>I11/SUM(Table3['#records])</f>
-        <v>0</v>
+        <v>0.27586206896551724</v>
       </c>
       <c r="L11">
         <v>5.5</v>
       </c>
       <c r="M11">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N11" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.82758620689655171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C12">
         <v>5</v>
       </c>
       <c r="D12">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>110</v>
@@ -7257,25 +8169,25 @@
         <f>COUNTIFS(Table2[QE R1:
 QE2/3/5/8],"ok",Table2[QE R2:
 cut-off],"reject")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="J12" s="9">
         <f>I12/SUM(Table3['#records])</f>
-        <v>1</v>
+        <v>0.27586206896551724</v>
       </c>
       <c r="L12">
         <v>5</v>
       </c>
       <c r="M12">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="N12" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.86206896551724133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C13">
         <v>5.5</v>
       </c>
@@ -7288,174 +8200,174 @@
       </c>
       <c r="M13">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="N13" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.86206896551724133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C14">
         <v>6</v>
       </c>
       <c r="D14">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L14">
         <v>4</v>
       </c>
       <c r="M14">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N14" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.89655172413793105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C15">
         <v>6.5</v>
       </c>
       <c r="D15">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15">
         <v>3.5</v>
       </c>
       <c r="M15">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="N15" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+        <v>0.89655172413793105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C16">
         <v>7</v>
       </c>
       <c r="D16">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L16">
         <v>3</v>
       </c>
       <c r="M16">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="N16" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="3:16" x14ac:dyDescent="0.25">
+        <v>0.93103448275862066</v>
+      </c>
+    </row>
+    <row r="17" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C17">
         <v>7.5</v>
       </c>
       <c r="D17">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L17">
         <v>2.5</v>
       </c>
       <c r="M17">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="N17" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="3:16" x14ac:dyDescent="0.25">
+        <v>0.93103448275862066</v>
+      </c>
+    </row>
+    <row r="18" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C18">
         <v>8</v>
       </c>
       <c r="D18">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L18">
         <v>2</v>
       </c>
       <c r="M18">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="N18" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="3:16" x14ac:dyDescent="0.25">
+        <v>0.93103448275862066</v>
+      </c>
+    </row>
+    <row r="19" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C19">
         <v>8.5</v>
       </c>
       <c r="D19">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L19">
         <v>1.5</v>
       </c>
       <c r="M19">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="N19" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="3:16" x14ac:dyDescent="0.25">
+        <v>0.93103448275862066</v>
+      </c>
+    </row>
+    <row r="20" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C20">
         <v>9</v>
       </c>
       <c r="D20">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L20">
         <v>1</v>
       </c>
       <c r="M20">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="N20" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="3:16" x14ac:dyDescent="0.25">
+        <v>0.93103448275862066</v>
+      </c>
+    </row>
+    <row r="21" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C21">
         <v>9.5</v>
       </c>
       <c r="D21">
         <f>COUNTIF(Table2[QE parsifal],Table3[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21">
         <v>0.5</v>
       </c>
       <c r="M21">
         <f>COUNTIF(Table2[QE parsifal],"&gt;=" &amp; Table5[[#This Row],[QE scores]])</f>
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="N21" s="9">
         <f>Table5[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="3:16" x14ac:dyDescent="0.25">
+        <v>0.93103448275862066</v>
+      </c>
+    </row>
+    <row r="22" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C22">
         <v>10</v>
       </c>
@@ -7475,7 +8387,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C23" s="6" t="s">
         <v>98</v>
       </c>
@@ -7485,15 +8397,15 @@
       </c>
       <c r="L23" s="6"/>
     </row>
-    <row r="24" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:16" x14ac:dyDescent="0.2">
       <c r="D24" s="5"/>
     </row>
-    <row r="25" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C25" s="3" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C27" s="3" t="s">
         <v>96</v>
       </c>
@@ -7528,19 +8440,19 @@
         <v>123</v>
       </c>
     </row>
-    <row r="28" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C28">
         <v>0</v>
       </c>
       <c r="D28">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E28" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F28" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
@@ -7548,42 +8460,42 @@
       </c>
       <c r="G28" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>1</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H28" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I28" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J28" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>1</v>
-      </c>
-      <c r="K28" s="13" t="e">
+        <v>0</v>
+      </c>
+      <c r="K28" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L28" s="12" t="e">
+        <v>1.796348381452564E-25</v>
+      </c>
+      <c r="L28" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M28" s="9" t="e">
+        <v>3.7723316010503847E-24</v>
+      </c>
+      <c r="M28" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
+        <v>1.7963483814525642E-25</v>
       </c>
       <c r="O28" s="4" t="s">
         <v>117</v>
       </c>
       <c r="P28" cm="1">
         <f t="array" ref="P28">SUM(Table37[QE scores]*Table37['#records])/$D$49</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="3:16" x14ac:dyDescent="0.25">
+        <v>8.0714285714285712</v>
+      </c>
+    </row>
+    <row r="29" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C29">
         <v>0.5</v>
       </c>
@@ -7595,44 +8507,44 @@
       <c r="E29" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F29" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H29" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I29" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J29" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K29" s="13" t="e">
+      <c r="K29" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L29" s="12" t="e">
+        <v>1.5546274617858815E-22</v>
+      </c>
+      <c r="L29" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M29" s="9" t="e">
+        <v>3.2647176697503511E-21</v>
+      </c>
+      <c r="M29" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
+        <v>1.5546274617858815E-22</v>
       </c>
       <c r="O29" s="4"/>
     </row>
-    <row r="30" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C30">
         <v>1</v>
       </c>
@@ -7644,46 +8556,46 @@
       <c r="E30" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F30" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G30" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H30" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I30" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K30" s="13" t="e">
+      <c r="K30" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L30" s="12" t="e">
+        <v>8.7315954626204478E-20</v>
+      </c>
+      <c r="L30" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M30" s="9" t="e">
+        <v>1.833635047150294E-18</v>
+      </c>
+      <c r="M30" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
+        <v>8.7315954626204478E-20</v>
       </c>
       <c r="O30" s="4" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="3:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C31">
         <v>1.5</v>
       </c>
@@ -7695,40 +8607,40 @@
       <c r="E31" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F31" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H31" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I31" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K31" s="13" t="e">
+      <c r="K31" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L31" s="12" t="e">
+        <v>3.1826756495701942E-17</v>
+      </c>
+      <c r="L31" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M31" s="9" t="e">
+        <v>6.6836188640974082E-16</v>
+      </c>
+      <c r="M31" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
+        <v>3.1826756495701942E-17</v>
       </c>
       <c r="O31" s="4" t="s">
         <v>117</v>
@@ -7736,10 +8648,10 @@
       <c r="P31">
         <f>AVERAGEIF(Table2[QE R1:
 QE2/3/5/8],"ok",Table2[QE score])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="3:16" x14ac:dyDescent="0.25">
+        <v>8.0714285714285712</v>
+      </c>
+    </row>
+    <row r="32" spans="3:16" x14ac:dyDescent="0.2">
       <c r="C32">
         <v>2</v>
       </c>
@@ -7751,40 +8663,40 @@
       <c r="E32" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F32" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H32" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I32" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J32" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K32" s="13" t="e">
+      <c r="K32" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L32" s="12" t="e">
+        <v>7.5287462467266207E-15</v>
+      </c>
+      <c r="L32" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M32" s="9" t="e">
+        <v>1.5810367118125904E-13</v>
+      </c>
+      <c r="M32" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
+        <v>7.5287462467266207E-15</v>
       </c>
       <c r="O32" s="4" t="s">
         <v>118</v>
@@ -7792,10 +8704,10 @@
       <c r="P32" cm="1">
         <f t="array" ref="P32">_xlfn.STDEV.P(IF(Table2[QE R1:
 QE2/3/5/8]="ok",Table2[QE score]))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="3:15" x14ac:dyDescent="0.25">
+        <v>0.7604152106033959</v>
+      </c>
+    </row>
+    <row r="33" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C33">
         <v>2.5</v>
       </c>
@@ -7807,43 +8719,43 @@
       <c r="E33" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F33" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H33" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I33" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K33" s="13" t="e">
+      <c r="K33" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L33" s="12" t="e">
+        <v>1.1558046606322563E-12</v>
+      </c>
+      <c r="L33" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M33" s="9" t="e">
+        <v>2.4271897873277382E-11</v>
+      </c>
+      <c r="M33" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="34" spans="3:15" x14ac:dyDescent="0.25">
+        <v>1.1558046606322563E-12</v>
+      </c>
+    </row>
+    <row r="34" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C34">
         <v>3</v>
       </c>
@@ -7855,46 +8767,46 @@
       <c r="E34" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F34" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G34" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H34" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I34" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J34" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K34" s="13" t="e">
+      <c r="K34" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L34" s="12" t="e">
+        <v>1.1515365483246049E-10</v>
+      </c>
+      <c r="L34" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M34" s="9" t="e">
+        <v>2.4182267514816703E-9</v>
+      </c>
+      <c r="M34" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
+        <v>1.1515365483246049E-10</v>
       </c>
       <c r="O34" s="4" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="35" spans="3:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C35">
         <v>3.5</v>
       </c>
@@ -7906,43 +8818,43 @@
       <c r="E35" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F35" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H35" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I35" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K35" s="13" t="e">
+      <c r="K35" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L35" s="12" t="e">
+        <v>7.4456482454290509E-9</v>
+      </c>
+      <c r="L35" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M35" s="9" t="e">
+        <v>1.5635861315401007E-7</v>
+      </c>
+      <c r="M35" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="36" spans="3:15" x14ac:dyDescent="0.25">
+        <v>7.4456482454290509E-9</v>
+      </c>
+    </row>
+    <row r="36" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C36">
         <v>4</v>
       </c>
@@ -7954,43 +8866,43 @@
       <c r="E36" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F36" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H36" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I36" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K36" s="13" t="e">
+      <c r="K36" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L36" s="12" t="e">
+        <v>3.124343726101338E-7</v>
+      </c>
+      <c r="L36" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M36" s="9" t="e">
+        <v>6.5611218248128096E-6</v>
+      </c>
+      <c r="M36" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="37" spans="3:15" x14ac:dyDescent="0.25">
+        <v>3.124343726101338E-7</v>
+      </c>
+    </row>
+    <row r="37" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C37">
         <v>4.5</v>
       </c>
@@ -8002,43 +8914,43 @@
       <c r="E37" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F37" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G37" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H37" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I37" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K37" s="13" t="e">
+      <c r="K37" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L37" s="12" t="e">
+        <v>8.508374597278666E-6</v>
+      </c>
+      <c r="L37" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M37" s="9" t="e">
+        <v>1.7867586654285198E-4</v>
+      </c>
+      <c r="M37" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="38" spans="3:15" x14ac:dyDescent="0.25">
+        <v>8.508374597278666E-6</v>
+      </c>
+    </row>
+    <row r="38" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C38">
         <v>5</v>
       </c>
@@ -8050,43 +8962,43 @@
       <c r="E38" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F38" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H38" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I38" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J38" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K38" s="13" t="e">
+      <c r="K38" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L38" s="12" t="e">
+        <v>1.5037162779309895E-4</v>
+      </c>
+      <c r="L38" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M38" s="9" t="e">
+        <v>3.1578041836550779E-3</v>
+      </c>
+      <c r="M38" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="39" spans="3:15" x14ac:dyDescent="0.25">
+        <v>1.5037162779309895E-4</v>
+      </c>
+    </row>
+    <row r="39" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C39">
         <v>5.5</v>
       </c>
@@ -8098,43 +9010,43 @@
       <c r="E39" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F39" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H39" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I39" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K39" s="13" t="e">
+      <c r="K39" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L39" s="12" t="e">
+        <v>1.724712469251695E-3</v>
+      </c>
+      <c r="L39" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M39" s="9" t="e">
+        <v>3.6218961854285595E-2</v>
+      </c>
+      <c r="M39" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="40" spans="3:15" x14ac:dyDescent="0.25">
+        <v>1.724712469251695E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C40">
         <v>6</v>
       </c>
@@ -8146,356 +9058,356 @@
       <c r="E40" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F40" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G40" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H40" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I40" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J40" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K40" s="13" t="e">
+      <c r="K40" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L40" s="12" t="e">
+        <v>1.2838048404294275E-2</v>
+      </c>
+      <c r="L40" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M40" s="9" t="e">
+        <v>0.26959901649017975</v>
+      </c>
+      <c r="M40" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="41" spans="3:15" x14ac:dyDescent="0.25">
+        <v>1.2838048404294275E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C41">
         <v>6.5</v>
       </c>
       <c r="D41">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E41" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="F41" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G41" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.72413793103448276</v>
       </c>
       <c r="H41" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="I41" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>4.7619047619047616E-2</v>
       </c>
       <c r="J41" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K41" s="13" t="e">
+        <v>4.7619047619047616E-2</v>
+      </c>
+      <c r="K41" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L41" s="12" t="e">
+        <v>6.2017294721938558E-2</v>
+      </c>
+      <c r="L41" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M41" s="9" t="e">
+        <v>1.3023631891607097</v>
+      </c>
+      <c r="M41" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="42" spans="3:15" x14ac:dyDescent="0.25">
+        <v>1.4398247102890938E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C42">
         <v>7</v>
       </c>
       <c r="D42">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E42" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="F42" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>0.95238095238095233</v>
       </c>
       <c r="G42" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.68965517241379315</v>
       </c>
       <c r="H42" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="I42" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="J42" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K42" s="13" t="e">
+        <v>9.5238095238095233E-2</v>
+      </c>
+      <c r="K42" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L42" s="12" t="e">
+        <v>0.19442769621071451</v>
+      </c>
+      <c r="L42" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M42" s="9" t="e">
+        <v>4.0829816204250049</v>
+      </c>
+      <c r="M42" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="43" spans="3:15" x14ac:dyDescent="0.25">
+        <v>9.918960097261928E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C43">
         <v>7.5</v>
       </c>
       <c r="D43">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E43" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F43" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="G43" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.62068965517241381</v>
       </c>
       <c r="H43" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="I43" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0.38095238095238093</v>
       </c>
       <c r="J43" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K43" s="13" t="e">
+        <v>0.23809523809523808</v>
+      </c>
+      <c r="K43" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L43" s="12" t="e">
+        <v>0.39558056464810687</v>
+      </c>
+      <c r="L43" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M43" s="9" t="e">
+        <v>8.3071918576102437</v>
+      </c>
+      <c r="M43" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="44" spans="3:15" x14ac:dyDescent="0.25">
+        <v>0.15748532655286876</v>
+      </c>
+    </row>
+    <row r="44" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C44">
         <v>8</v>
       </c>
       <c r="D44">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E44" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F44" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>0.61904761904761907</v>
       </c>
       <c r="G44" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.44827586206896552</v>
       </c>
       <c r="H44" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="I44" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0.52380952380952384</v>
       </c>
       <c r="J44" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K44" s="13" t="e">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="K44" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L44" s="12" t="e">
+        <v>0.52232794942481031</v>
+      </c>
+      <c r="L44" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M44" s="9" t="e">
+        <v>10.968886937921017</v>
+      </c>
+      <c r="M44" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="45" spans="3:15" x14ac:dyDescent="0.25">
+        <v>0.37947080656766746</v>
+      </c>
+    </row>
+    <row r="45" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C45">
         <v>8.5</v>
       </c>
       <c r="D45">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E45" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F45" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>0.47619047619047616</v>
       </c>
       <c r="G45" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.34482758620689657</v>
       </c>
       <c r="H45" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="I45" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0.80952380952380953</v>
       </c>
       <c r="J45" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K45" s="13" t="e">
+        <v>0.2857142857142857</v>
+      </c>
+      <c r="K45" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L45" s="12" t="e">
+        <v>0.44759279596826385</v>
+      </c>
+      <c r="L45" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M45" s="9" t="e">
+        <v>9.3994487153335413</v>
+      </c>
+      <c r="M45" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="46" spans="3:15" x14ac:dyDescent="0.25">
+        <v>0.16187851025397815</v>
+      </c>
+    </row>
+    <row r="46" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C46">
         <v>9</v>
       </c>
       <c r="D46">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E46" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F46" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>0.19047619047619047</v>
       </c>
       <c r="G46" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>0.13793103448275862</v>
       </c>
       <c r="H46" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="I46" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
-        <v>1</v>
+        <v>0.95238095238095233</v>
       </c>
       <c r="J46" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K46" s="13" t="e">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="K46" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L46" s="12" t="e">
+        <v>0.24891691737552185</v>
+      </c>
+      <c r="L46" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M46" s="9" t="e">
+        <v>5.2272552648859589</v>
+      </c>
+      <c r="M46" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="47" spans="3:15" x14ac:dyDescent="0.25">
+        <v>0.106059774518379</v>
+      </c>
+    </row>
+    <row r="47" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C47">
         <v>9.5</v>
       </c>
       <c r="D47">
         <f>COUNTIFS(Table2[QE parsifal],Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" s="5">
         <f>COUNTIFS(Table2[QE parsifal],"&gt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F47" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$49</f>
-        <v>0</v>
+        <v>4.7619047619047616E-2</v>
       </c>
       <c r="G47" s="9">
         <f>Table37[[#This Row],[cumul '#]]/$D$23</f>
-        <v>0</v>
+        <v>3.4482758620689655E-2</v>
       </c>
       <c r="H47" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="I47" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
@@ -8503,22 +9415,22 @@
       </c>
       <c r="J47" s="13">
         <f>Table37[[#This Row],['#records]]/$D$49</f>
-        <v>0</v>
-      </c>
-      <c r="K47" s="13" t="e">
+        <v>4.7619047619047616E-2</v>
+      </c>
+      <c r="K47" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L47" s="12" t="e">
+        <v>8.9837414274778066E-2</v>
+      </c>
+      <c r="L47" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M47" s="9" t="e">
+        <v>1.8865856997703394</v>
+      </c>
+      <c r="M47" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="48" spans="3:15" x14ac:dyDescent="0.25">
+        <v>4.2218366655730449E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="3:15" x14ac:dyDescent="0.2">
       <c r="C48">
         <v>10</v>
       </c>
@@ -8543,7 +9455,7 @@
       <c r="H48" s="12">
         <f>COUNTIFS(Table2[QE parsifal],"&lt;=" &amp; Table37[[#This Row],[QE scores]],Table2[QE R1:
 QE2/3/5/8],"ok")</f>
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="I48" s="9">
         <f>Table37[[#This Row],[inv cuml '#]]/$D$49</f>
@@ -8553,38 +9465,38 @@
         <f>Table37[[#This Row],['#records]]/$D$49</f>
         <v>0</v>
       </c>
-      <c r="K48" s="13" t="e">
+      <c r="K48" s="13">
         <f>_xlfn.NORM.DIST(Table37[[#This Row],[QE scores]],$P$31,$P$32,FALSE)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="L48" s="12" t="e">
+        <v>2.1042220941051924E-2</v>
+      </c>
+      <c r="L48" s="12">
         <f>Table37[[#This Row],[^Y]]*$D$49</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="M48" s="9" t="e">
+        <v>0.44188663976209042</v>
+      </c>
+      <c r="M48" s="9">
         <f>(Table37[[#This Row],[^'#records]]-Table37[[#This Row],['#records]])/$D$49</f>
-        <v>#NUM!</v>
-      </c>
-    </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.25">
+        <v>2.1042220941051924E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C49" s="6" t="s">
         <v>98</v>
       </c>
       <c r="D49" s="5">
         <f>SUM(Table37['#records])</f>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="50" spans="3:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="50" spans="3:6" x14ac:dyDescent="0.2">
       <c r="C50" s="6" t="s">
         <v>116</v>
       </c>
       <c r="D50">
         <f>$D$23-$D$49</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="52" spans="3:6" x14ac:dyDescent="0.2">
       <c r="F52" s="9"/>
     </row>
   </sheetData>
@@ -8603,9 +9515,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41055AAB-D91C-4300-A0FB-8A5F79915C25}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="4.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="4.7109375" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="4.6640625" style="4"/>
+    <col min="1" max="16384" width="4.7109375" style="4"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>